<commit_message>
update mapping to new template in modern mode
</commit_message>
<xml_diff>
--- a/template/template.xlsx
+++ b/template/template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tuong Minh\Xuất hình ảnh thí sinh\digital-certificate-excel-mapping-tool\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tuong Minh\CFLA Software\digital-certificate-excel-mapping-tool\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C8A06B-7293-41CB-8D20-232A56D6EC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A98899D-A5AF-4007-9644-56175C0FE823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -150,7 +150,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U2" authorId="3" shapeId="0" xr:uid="{D752925C-48BB-47B5-84EB-921F5C93C2DA}">
+    <comment ref="R2" authorId="3" shapeId="0" xr:uid="{D752925C-48BB-47B5-84EB-921F5C93C2DA}">
       <text>
         <r>
           <rPr>
@@ -171,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z2" authorId="4" shapeId="0" xr:uid="{16451AA9-07BF-464D-93E1-48687E056383}">
+    <comment ref="W2" authorId="4" shapeId="0" xr:uid="{16451AA9-07BF-464D-93E1-48687E056383}">
       <text>
         <r>
           <rPr>
@@ -192,7 +192,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC2" authorId="5" shapeId="0" xr:uid="{31B64C8A-4B99-4AAF-8D2E-5C749DD02EA6}">
+    <comment ref="Z2" authorId="5" shapeId="0" xr:uid="{31B64C8A-4B99-4AAF-8D2E-5C749DD02EA6}">
       <text>
         <r>
           <rPr>
@@ -218,7 +218,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="429">
   <si>
     <t>HƯỚNG DẪN NHẬP THÔNG TIN</t>
   </si>
@@ -442,46 +442,13 @@
     <t>Địa danh nơi cơ quan cấp chứng chỉ đặt trụ sở</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>0041036</t>
-  </si>
-  <si>
-    <t>02108/CTU0009.31425</t>
-  </si>
-  <si>
-    <t>Chứng chỉ ngoại ngữ Bậc 3</t>
-  </si>
-  <si>
-    <t>Nguyễn Trần Trúc Duy</t>
-  </si>
-  <si>
-    <t>18/06/1994</t>
-  </si>
-  <si>
     <t>Nam</t>
   </si>
   <si>
     <t>Kinh</t>
   </si>
   <si>
-    <t>Tiền Giang</t>
-  </si>
-  <si>
-    <t>Trường Đại học Cần Thơ</t>
-  </si>
-  <si>
     <t>Thành phố Cần Thơ</t>
-  </si>
-  <si>
-    <t>08/04/2025</t>
-  </si>
-  <si>
-    <t>Hiệu Trưởng</t>
-  </si>
-  <si>
-    <t>Trần Trung Tính</t>
   </si>
   <si>
     <t>Đã số hóa đầy đủ, chính xác</t>
@@ -1622,9 +1589,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\/mm\/yyyy"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -1799,7 +1765,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1913,19 +1879,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2580,7 +2533,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AL16"/>
+  <dimension ref="A1:AI15"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="8" style="24" customWidth="1"/>
@@ -2598,23 +2551,20 @@
     <col min="13" max="13" width="21.44140625" style="25" customWidth="1"/>
     <col min="14" max="14" width="29.44140625" style="25" customWidth="1"/>
     <col min="15" max="15" width="15.33203125" style="25" customWidth="1"/>
-    <col min="16" max="16" width="25.5546875" style="25" customWidth="1"/>
-    <col min="17" max="17" width="15.5546875" style="25" customWidth="1"/>
-    <col min="18" max="18" width="15.33203125" style="25" customWidth="1"/>
-    <col min="19" max="19" width="20.33203125" style="25" customWidth="1"/>
-    <col min="20" max="20" width="15.44140625" style="25" customWidth="1"/>
-    <col min="21" max="21" width="31.44140625" style="25" customWidth="1"/>
-    <col min="22" max="22" width="15.44140625" style="25" customWidth="1"/>
-    <col min="23" max="23" width="19.109375" style="24" customWidth="1"/>
-    <col min="24" max="25" width="19.44140625" style="26" customWidth="1"/>
-    <col min="26" max="27" width="21.109375" style="27" customWidth="1"/>
-    <col min="28" max="28" width="29.88671875" style="28" customWidth="1"/>
-    <col min="29" max="29" width="29.44140625" style="25" customWidth="1"/>
-    <col min="30" max="30" width="8.88671875" style="1" customWidth="1"/>
-    <col min="31" max="16384" width="8.88671875" style="1"/>
+    <col min="16" max="16" width="20.33203125" style="25" customWidth="1"/>
+    <col min="17" max="17" width="15.44140625" style="25" customWidth="1"/>
+    <col min="18" max="18" width="31.44140625" style="25" customWidth="1"/>
+    <col min="19" max="19" width="15.44140625" style="25" customWidth="1"/>
+    <col min="20" max="20" width="19.109375" style="24" customWidth="1"/>
+    <col min="21" max="22" width="19.44140625" style="26" customWidth="1"/>
+    <col min="23" max="24" width="21.109375" style="27" customWidth="1"/>
+    <col min="25" max="25" width="29.88671875" style="28" customWidth="1"/>
+    <col min="26" max="26" width="29.44140625" style="25" customWidth="1"/>
+    <col min="27" max="27" width="8.88671875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="3" customFormat="1" ht="35.1" customHeight="1">
+    <row r="1" spans="1:35" s="3" customFormat="1" ht="35.1" customHeight="1">
       <c r="A1" s="39" t="s">
         <v>44</v>
       </c>
@@ -2643,20 +2593,17 @@
       <c r="X1" s="39"/>
       <c r="Y1" s="39"/>
       <c r="Z1" s="39"/>
-      <c r="AA1" s="39"/>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="39"/>
-      <c r="AD1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="29"/>
+      <c r="AD1" s="30"/>
       <c r="AE1" s="1"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="30"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
       <c r="AH1" s="1"/>
       <c r="AI1" s="1"/>
-      <c r="AJ1" s="1"/>
-      <c r="AK1" s="1"/>
-      <c r="AL1" s="1"/>
-    </row>
-    <row r="2" spans="1:38" s="3" customFormat="1" ht="35.1" customHeight="1">
+    </row>
+    <row r="2" spans="1:35" s="3" customFormat="1" ht="35.1" customHeight="1">
       <c r="A2" s="31" t="s">
         <v>2</v>
       </c>
@@ -2703,130 +2650,56 @@
         <v>29</v>
       </c>
       <c r="P2" s="31" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="Q2" s="31" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="R2" s="31" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="S2" s="31" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="T2" s="31" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="U2" s="31" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="V2" s="31" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="W2" s="31" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="X2" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="Y2" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z2" s="31" t="s">
-        <v>40</v>
-      </c>
-      <c r="AA2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="AB2" s="32" t="s">
+      <c r="Y2" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="AC2" s="32" t="s">
+      <c r="Z2" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="AD2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="29"/>
+      <c r="AD2" s="30"/>
       <c r="AE2" s="1"/>
-      <c r="AF2" s="29"/>
-      <c r="AG2" s="30"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
       <c r="AH2" s="1"/>
       <c r="AI2" s="1"/>
-      <c r="AJ2" s="1"/>
-      <c r="AK2" s="1"/>
-      <c r="AL2" s="1"/>
-    </row>
-    <row r="3" spans="1:38">
-      <c r="A3" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="34" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" s="41" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="34" t="s">
+    </row>
+    <row r="15" spans="1:35">
+      <c r="E15" s="25" t="s">
         <v>52</v>
-      </c>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41" t="s">
-        <v>53</v>
-      </c>
-      <c r="J3" s="42" t="s">
-        <v>54</v>
-      </c>
-      <c r="K3" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="L3" s="41"/>
-      <c r="M3" s="43" t="s">
-        <v>56</v>
-      </c>
-      <c r="N3" s="41"/>
-      <c r="O3" s="42"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="42"/>
-      <c r="S3" s="44">
-        <v>5.5</v>
-      </c>
-      <c r="T3" s="41" t="s">
-        <v>57</v>
-      </c>
-      <c r="U3" s="41" t="s">
-        <v>58</v>
-      </c>
-      <c r="V3" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="W3" s="41" t="s">
-        <v>57</v>
-      </c>
-      <c r="X3" s="41" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y3" s="41" t="s">
-        <v>61</v>
-      </c>
-      <c r="Z3" s="41"/>
-      <c r="AA3" s="45"/>
-      <c r="AB3" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="AC3" s="42"/>
-    </row>
-    <row r="16" spans="1:38">
-      <c r="E16" s="25" t="s">
-        <v>63</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A1:Z1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2834,23 +2707,23 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000000000000}">
-          <x14:formula1>
-            <xm:f>DanhMuc!$B$4:$B$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>J3:J1999</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
             <xm:f>DanhMuc!$V$4:$V$7</xm:f>
           </x14:formula1>
-          <xm:sqref>W4:W1999</xm:sqref>
+          <xm:sqref>T3:T1998</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000002000000}">
           <x14:formula1>
             <xm:f>DanhMuc!$S$4:$S$6</xm:f>
           </x14:formula1>
-          <xm:sqref>Y4:Y1999</xm:sqref>
+          <xm:sqref>V3:V1998</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000000000000}">
+          <x14:formula1>
+            <xm:f>DanhMuc!$B$4:$B$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>J3:J1998</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2874,84 +2747,84 @@
   <sheetData>
     <row r="1" spans="1:22" ht="32.25" customHeight="1">
       <c r="A1" s="40" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B1" s="40"/>
       <c r="D1" s="40" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="E1" s="40"/>
       <c r="F1" s="40"/>
       <c r="H1" s="40" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="I1" s="40"/>
       <c r="J1" s="40"/>
       <c r="L1" s="40" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="M1" s="40"/>
       <c r="O1" s="40" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="P1" s="40"/>
       <c r="R1" s="40" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="S1" s="40"/>
       <c r="U1" s="40" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="V1" s="40"/>
     </row>
     <row r="3" spans="1:22" ht="14.25" customHeight="1">
       <c r="A3" s="33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="B3" s="33" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="D3" s="33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="F3" s="33" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="H3" s="33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="I3" s="33" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="J3" s="33" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="L3" s="33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="M3" s="33" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="O3" s="33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="P3" s="33" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="R3" s="33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="S3" s="33" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="U3" s="33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="V3" s="33" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -2959,45 +2832,45 @@
         <v>1</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D4" s="34">
         <v>1</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="F4" s="34"/>
       <c r="H4" s="34">
         <v>1</v>
       </c>
       <c r="I4" s="35" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="J4" s="34"/>
       <c r="L4" s="34">
         <v>1</v>
       </c>
       <c r="M4" s="35" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="O4" s="34">
         <v>1</v>
       </c>
       <c r="P4" s="35" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="R4" s="34">
         <v>1</v>
       </c>
       <c r="S4" s="35" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="U4" s="34">
         <v>1</v>
       </c>
       <c r="V4" s="35" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -3005,47 +2878,47 @@
         <v>2</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="D5" s="34">
         <v>2</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="F5" s="34"/>
       <c r="H5" s="34">
         <v>2</v>
       </c>
       <c r="I5" s="35" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="J5" s="34" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="L5" s="34">
         <v>2</v>
       </c>
       <c r="M5" s="35" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="O5" s="34">
         <v>2</v>
       </c>
       <c r="P5" s="35" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="R5" s="34">
         <v>2</v>
       </c>
       <c r="S5" s="35" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="U5" s="34">
         <v>2</v>
       </c>
       <c r="V5" s="35" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -3053,47 +2926,47 @@
         <v>3</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="D6" s="34">
         <v>3</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="F6" s="34"/>
       <c r="H6" s="34">
         <v>3</v>
       </c>
       <c r="I6" s="35" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="J6" s="34" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="L6" s="34">
         <v>3</v>
       </c>
       <c r="M6" s="35" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="O6" s="34">
         <v>3</v>
       </c>
       <c r="P6" s="35" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="R6" s="34">
         <v>3</v>
       </c>
       <c r="S6" s="35" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="U6" s="34">
         <v>3</v>
       </c>
       <c r="V6" s="35" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -3101,35 +2974,35 @@
         <v>4</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="F7" s="34"/>
       <c r="H7" s="34">
         <v>4</v>
       </c>
       <c r="I7" s="35" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J7" s="34" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L7" s="34">
         <v>4</v>
       </c>
       <c r="M7" s="35" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="O7" s="34">
         <v>4</v>
       </c>
       <c r="P7" s="35" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="U7" s="34">
         <v>4</v>
       </c>
       <c r="V7" s="35" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:22">
@@ -3137,29 +3010,29 @@
         <v>5</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="F8" s="34"/>
       <c r="H8" s="34">
         <v>5</v>
       </c>
       <c r="I8" s="35" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="J8" s="34" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="L8" s="34">
         <v>5</v>
       </c>
       <c r="M8" s="35" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="O8" s="34">
         <v>5</v>
       </c>
       <c r="P8" s="35" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -3167,29 +3040,29 @@
         <v>6</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="F9" s="34"/>
       <c r="H9" s="34">
         <v>6</v>
       </c>
       <c r="I9" s="35" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="J9" s="34" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="L9" s="34">
         <v>6</v>
       </c>
       <c r="M9" s="35" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="O9" s="34">
         <v>6</v>
       </c>
       <c r="P9" s="35" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -3197,29 +3070,29 @@
         <v>7</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="F10" s="34"/>
       <c r="H10" s="34">
         <v>7</v>
       </c>
       <c r="I10" s="35" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="J10" s="34" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="L10" s="34">
         <v>7</v>
       </c>
       <c r="M10" s="35" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="O10" s="34">
         <v>7</v>
       </c>
       <c r="P10" s="35" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -3227,27 +3100,27 @@
         <v>8</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="F11" s="34"/>
       <c r="H11" s="34">
         <v>8</v>
       </c>
       <c r="I11" s="35" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J11" s="34"/>
       <c r="L11" s="34">
         <v>8</v>
       </c>
       <c r="M11" s="35" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="O11" s="34">
         <v>8</v>
       </c>
       <c r="P11" s="35" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:22">
@@ -3255,29 +3128,29 @@
         <v>9</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="F12" s="34"/>
       <c r="H12" s="34">
         <v>9</v>
       </c>
       <c r="I12" s="35" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="J12" s="34" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="L12" s="34">
         <v>9</v>
       </c>
       <c r="M12" s="35" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="O12" s="34">
         <v>9</v>
       </c>
       <c r="P12" s="35" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -3285,27 +3158,27 @@
         <v>10</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F13" s="34"/>
       <c r="H13" s="34">
         <v>10</v>
       </c>
       <c r="I13" s="35" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="J13" s="34"/>
       <c r="L13" s="34">
         <v>10</v>
       </c>
       <c r="M13" s="35" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="O13" s="34">
         <v>10</v>
       </c>
       <c r="P13" s="35" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:22">
@@ -3313,29 +3186,29 @@
         <v>11</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="F14" s="34"/>
       <c r="H14" s="34">
         <v>11</v>
       </c>
       <c r="I14" s="35" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="J14" s="34" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="L14" s="34">
         <v>11</v>
       </c>
       <c r="M14" s="35" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="O14" s="34">
         <v>11</v>
       </c>
       <c r="P14" s="35" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -3343,29 +3216,29 @@
         <v>12</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="F15" s="34"/>
       <c r="H15" s="34">
         <v>12</v>
       </c>
       <c r="I15" s="35" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="J15" s="34" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="L15" s="34">
         <v>12</v>
       </c>
       <c r="M15" s="35" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="O15" s="34">
         <v>12</v>
       </c>
       <c r="P15" s="35" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -3373,29 +3246,29 @@
         <v>13</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="F16" s="34"/>
       <c r="H16" s="34">
         <v>13</v>
       </c>
       <c r="I16" s="35" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="J16" s="34" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="L16" s="34">
         <v>13</v>
       </c>
       <c r="M16" s="35" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="O16" s="34">
         <v>13</v>
       </c>
       <c r="P16" s="35" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="4:16">
@@ -3403,27 +3276,27 @@
         <v>14</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="F17" s="34"/>
       <c r="H17" s="34">
         <v>14</v>
       </c>
       <c r="I17" s="35" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="J17" s="34"/>
       <c r="L17" s="34">
         <v>14</v>
       </c>
       <c r="M17" s="35" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="O17" s="34">
         <v>14</v>
       </c>
       <c r="P17" s="35" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" spans="4:16">
@@ -3431,27 +3304,27 @@
         <v>15</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="F18" s="34"/>
       <c r="H18" s="34">
         <v>15</v>
       </c>
       <c r="I18" s="35" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="J18" s="34"/>
       <c r="L18" s="34">
         <v>15</v>
       </c>
       <c r="M18" s="35" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="O18" s="34">
         <v>15</v>
       </c>
       <c r="P18" s="35" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="4:16">
@@ -3459,29 +3332,29 @@
         <v>16</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="F19" s="34"/>
       <c r="H19" s="34">
         <v>16</v>
       </c>
       <c r="I19" s="35" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="J19" s="34" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="L19" s="34">
         <v>16</v>
       </c>
       <c r="M19" s="35" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O19" s="34">
         <v>16</v>
       </c>
       <c r="P19" s="35" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" spans="4:16">
@@ -3489,29 +3362,29 @@
         <v>17</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="F20" s="34"/>
       <c r="H20" s="34">
         <v>17</v>
       </c>
       <c r="I20" s="35" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="J20" s="34" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="L20" s="34">
         <v>17</v>
       </c>
       <c r="M20" s="35" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O20" s="34">
         <v>17</v>
       </c>
       <c r="P20" s="35" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="4:16">
@@ -3519,29 +3392,29 @@
         <v>18</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="F21" s="34"/>
       <c r="H21" s="34">
         <v>18</v>
       </c>
       <c r="I21" s="35" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="J21" s="34" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="L21" s="34">
         <v>18</v>
       </c>
       <c r="M21" s="35" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="O21" s="34">
         <v>18</v>
       </c>
       <c r="P21" s="35" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" spans="4:16">
@@ -3549,29 +3422,29 @@
         <v>19</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F22" s="34"/>
       <c r="H22" s="34">
         <v>19</v>
       </c>
       <c r="I22" s="35" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="J22" s="34" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="L22" s="34">
         <v>19</v>
       </c>
       <c r="M22" s="35" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="O22" s="34">
         <v>19</v>
       </c>
       <c r="P22" s="35" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" spans="4:16">
@@ -3579,29 +3452,29 @@
         <v>20</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="F23" s="34"/>
       <c r="H23" s="34">
         <v>20</v>
       </c>
       <c r="I23" s="35" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="J23" s="34" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="L23" s="34">
         <v>20</v>
       </c>
       <c r="M23" s="35" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="O23" s="34">
         <v>20</v>
       </c>
       <c r="P23" s="35" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" spans="4:16">
@@ -3609,29 +3482,29 @@
         <v>21</v>
       </c>
       <c r="E24" s="35" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="F24" s="34"/>
       <c r="H24" s="34">
         <v>21</v>
       </c>
       <c r="I24" s="35" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="J24" s="34" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="L24" s="34">
         <v>21</v>
       </c>
       <c r="M24" s="35" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="O24" s="34">
         <v>21</v>
       </c>
       <c r="P24" s="35" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="4:16">
@@ -3639,27 +3512,27 @@
         <v>22</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="F25" s="34"/>
       <c r="H25" s="34">
         <v>22</v>
       </c>
       <c r="I25" s="35" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="J25" s="34"/>
       <c r="L25" s="34">
         <v>22</v>
       </c>
       <c r="M25" s="35" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="O25" s="34">
         <v>22</v>
       </c>
       <c r="P25" s="35" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26" spans="4:16">
@@ -3667,29 +3540,29 @@
         <v>23</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="F26" s="34"/>
       <c r="H26" s="34">
         <v>23</v>
       </c>
       <c r="I26" s="35" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="J26" s="34" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="L26" s="34">
         <v>23</v>
       </c>
       <c r="M26" s="35" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="O26" s="34">
         <v>23</v>
       </c>
       <c r="P26" s="35" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27" spans="4:16">
@@ -3697,29 +3570,29 @@
         <v>24</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="F27" s="34"/>
       <c r="H27" s="34">
         <v>24</v>
       </c>
       <c r="I27" s="35" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="J27" s="34" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="L27" s="34">
         <v>24</v>
       </c>
       <c r="M27" s="35" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="O27" s="34">
         <v>24</v>
       </c>
       <c r="P27" s="35" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28" spans="4:16">
@@ -3727,29 +3600,29 @@
         <v>25</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="F28" s="34"/>
       <c r="H28" s="34">
         <v>25</v>
       </c>
       <c r="I28" s="35" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="J28" s="34" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="L28" s="34">
         <v>25</v>
       </c>
       <c r="M28" s="35" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="O28" s="34">
         <v>25</v>
       </c>
       <c r="P28" s="35" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" spans="4:16">
@@ -3757,29 +3630,29 @@
         <v>26</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="F29" s="34"/>
       <c r="H29" s="34">
         <v>26</v>
       </c>
       <c r="I29" s="35" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="J29" s="34" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="L29" s="34">
         <v>26</v>
       </c>
       <c r="M29" s="35" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="O29" s="34">
         <v>26</v>
       </c>
       <c r="P29" s="35" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="4:16">
@@ -3787,29 +3660,29 @@
         <v>27</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="F30" s="34"/>
       <c r="H30" s="34">
         <v>27</v>
       </c>
       <c r="I30" s="35" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="J30" s="34" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="L30" s="34">
         <v>27</v>
       </c>
       <c r="M30" s="35" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="O30" s="34">
         <v>27</v>
       </c>
       <c r="P30" s="35" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" spans="4:16">
@@ -3817,29 +3690,29 @@
         <v>28</v>
       </c>
       <c r="E31" s="35" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="F31" s="34"/>
       <c r="H31" s="34">
         <v>28</v>
       </c>
       <c r="I31" s="35" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="J31" s="34" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="L31" s="34">
         <v>28</v>
       </c>
       <c r="M31" s="35" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="O31" s="34">
         <v>28</v>
       </c>
       <c r="P31" s="35" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
     </row>
     <row r="32" spans="4:16">
@@ -3847,29 +3720,29 @@
         <v>29</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="F32" s="34"/>
       <c r="H32" s="34">
         <v>29</v>
       </c>
       <c r="I32" s="35" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="J32" s="34" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="L32" s="34">
         <v>29</v>
       </c>
       <c r="M32" s="35" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="O32" s="34">
         <v>29</v>
       </c>
       <c r="P32" s="35" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
     </row>
     <row r="33" spans="4:16">
@@ -3877,29 +3750,29 @@
         <v>30</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="F33" s="34"/>
       <c r="H33" s="34">
         <v>30</v>
       </c>
       <c r="I33" s="35" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="J33" s="34" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="L33" s="34">
         <v>30</v>
       </c>
       <c r="M33" s="35" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="O33" s="34">
         <v>30</v>
       </c>
       <c r="P33" s="35" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34" spans="4:16">
@@ -3907,29 +3780,29 @@
         <v>31</v>
       </c>
       <c r="E34" s="35" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="F34" s="34"/>
       <c r="H34" s="34">
         <v>31</v>
       </c>
       <c r="I34" s="35" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="J34" s="34" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="L34" s="34">
         <v>31</v>
       </c>
       <c r="M34" s="35" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="O34" s="34">
         <v>31</v>
       </c>
       <c r="P34" s="35" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
     </row>
     <row r="35" spans="4:16">
@@ -3937,27 +3810,27 @@
         <v>32</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="F35" s="34"/>
       <c r="H35" s="34">
         <v>32</v>
       </c>
       <c r="I35" s="35" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="J35" s="34"/>
       <c r="L35" s="34">
         <v>32</v>
       </c>
       <c r="M35" s="35" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="O35" s="34">
         <v>32</v>
       </c>
       <c r="P35" s="35" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
     </row>
     <row r="36" spans="4:16">
@@ -3965,29 +3838,29 @@
         <v>33</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="F36" s="34"/>
       <c r="H36" s="34">
         <v>33</v>
       </c>
       <c r="I36" s="35" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="J36" s="34" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="L36" s="34">
         <v>33</v>
       </c>
       <c r="M36" s="35" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="O36" s="34">
         <v>33</v>
       </c>
       <c r="P36" s="35" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
     </row>
     <row r="37" spans="4:16">
@@ -3995,29 +3868,29 @@
         <v>34</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="F37" s="34"/>
       <c r="H37" s="34">
         <v>34</v>
       </c>
       <c r="I37" s="35" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="J37" s="34" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="L37" s="34">
         <v>34</v>
       </c>
       <c r="M37" s="35" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="O37" s="34">
         <v>34</v>
       </c>
       <c r="P37" s="35" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
     </row>
     <row r="38" spans="4:16">
@@ -4025,29 +3898,29 @@
         <v>35</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="F38" s="34"/>
       <c r="H38" s="34">
         <v>35</v>
       </c>
       <c r="I38" s="35" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="J38" s="34" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="L38" s="34">
         <v>35</v>
       </c>
       <c r="M38" s="35" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="O38" s="34">
         <v>35</v>
       </c>
       <c r="P38" s="35" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
     </row>
     <row r="39" spans="4:16">
@@ -4055,23 +3928,23 @@
         <v>36</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="F39" s="34"/>
       <c r="H39" s="34">
         <v>36</v>
       </c>
       <c r="I39" s="35" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="J39" s="34" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="L39" s="34">
         <v>36</v>
       </c>
       <c r="M39" s="35" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="40" spans="4:16">
@@ -4079,23 +3952,23 @@
         <v>37</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F40" s="34"/>
       <c r="H40" s="34">
         <v>37</v>
       </c>
       <c r="I40" s="35" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="J40" s="34" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="L40" s="34">
         <v>37</v>
       </c>
       <c r="M40" s="35" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
     </row>
     <row r="41" spans="4:16">
@@ -4103,23 +3976,23 @@
         <v>38</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="F41" s="34"/>
       <c r="H41" s="34">
         <v>38</v>
       </c>
       <c r="I41" s="35" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="J41" s="34" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="L41" s="34">
         <v>38</v>
       </c>
       <c r="M41" s="35" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
     </row>
     <row r="42" spans="4:16">
@@ -4127,23 +4000,23 @@
         <v>39</v>
       </c>
       <c r="E42" s="35" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="F42" s="34"/>
       <c r="H42" s="34">
         <v>39</v>
       </c>
       <c r="I42" s="35" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="J42" s="34" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="L42" s="34">
         <v>39</v>
       </c>
       <c r="M42" s="35" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
     </row>
     <row r="43" spans="4:16">
@@ -4151,23 +4024,23 @@
         <v>40</v>
       </c>
       <c r="E43" s="35" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="F43" s="34"/>
       <c r="H43" s="34">
         <v>40</v>
       </c>
       <c r="I43" s="35" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="J43" s="34" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="L43" s="34">
         <v>40</v>
       </c>
       <c r="M43" s="35" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
     </row>
     <row r="44" spans="4:16">
@@ -4175,21 +4048,21 @@
         <v>41</v>
       </c>
       <c r="E44" s="35" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="F44" s="34"/>
       <c r="H44" s="34">
         <v>41</v>
       </c>
       <c r="I44" s="35" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="J44" s="34"/>
       <c r="L44" s="34">
         <v>41</v>
       </c>
       <c r="M44" s="35" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
     </row>
     <row r="45" spans="4:16">
@@ -4197,23 +4070,23 @@
         <v>42</v>
       </c>
       <c r="E45" s="35" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="F45" s="34"/>
       <c r="H45" s="34">
         <v>42</v>
       </c>
       <c r="I45" s="35" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="J45" s="34" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="L45" s="34">
         <v>42</v>
       </c>
       <c r="M45" s="35" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" spans="4:16">
@@ -4221,23 +4094,23 @@
         <v>43</v>
       </c>
       <c r="E46" s="35" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="F46" s="34"/>
       <c r="H46" s="34">
         <v>43</v>
       </c>
       <c r="I46" s="35" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="J46" s="34" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="L46" s="34">
         <v>43</v>
       </c>
       <c r="M46" s="35" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
     </row>
     <row r="47" spans="4:16">
@@ -4245,23 +4118,23 @@
         <v>44</v>
       </c>
       <c r="E47" s="35" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="F47" s="34"/>
       <c r="H47" s="34">
         <v>44</v>
       </c>
       <c r="I47" s="35" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="J47" s="34" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="L47" s="34">
         <v>44</v>
       </c>
       <c r="M47" s="35" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="4:16">
@@ -4269,21 +4142,21 @@
         <v>45</v>
       </c>
       <c r="E48" s="35" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="F48" s="34"/>
       <c r="H48" s="34">
         <v>45</v>
       </c>
       <c r="I48" s="35" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="J48" s="34"/>
       <c r="L48" s="34">
         <v>45</v>
       </c>
       <c r="M48" s="35" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
     </row>
     <row r="49" spans="4:13">
@@ -4291,23 +4164,23 @@
         <v>46</v>
       </c>
       <c r="E49" s="35" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="F49" s="34"/>
       <c r="H49" s="34">
         <v>46</v>
       </c>
       <c r="I49" s="35" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="J49" s="34" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="L49" s="34">
         <v>46</v>
       </c>
       <c r="M49" s="35" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50" spans="4:13">
@@ -4315,23 +4188,23 @@
         <v>47</v>
       </c>
       <c r="E50" s="35" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="F50" s="34"/>
       <c r="H50" s="34">
         <v>47</v>
       </c>
       <c r="I50" s="35" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="J50" s="34" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="L50" s="34">
         <v>47</v>
       </c>
       <c r="M50" s="35" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51" spans="4:13">
@@ -4339,23 +4212,23 @@
         <v>48</v>
       </c>
       <c r="E51" s="35" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="F51" s="34"/>
       <c r="H51" s="34">
         <v>48</v>
       </c>
       <c r="I51" s="35" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="J51" s="34" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="L51" s="34">
         <v>48</v>
       </c>
       <c r="M51" s="35" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
     </row>
     <row r="52" spans="4:13">
@@ -4363,23 +4236,23 @@
         <v>49</v>
       </c>
       <c r="E52" s="35" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="F52" s="34"/>
       <c r="H52" s="34">
         <v>49</v>
       </c>
       <c r="I52" s="35" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="J52" s="34" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="L52" s="34">
         <v>49</v>
       </c>
       <c r="M52" s="35" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
     </row>
     <row r="53" spans="4:13">
@@ -4387,23 +4260,23 @@
         <v>50</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="F53" s="34"/>
       <c r="H53" s="34">
         <v>50</v>
       </c>
       <c r="I53" s="35" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="J53" s="34" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="L53" s="34">
         <v>50</v>
       </c>
       <c r="M53" s="35" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
     </row>
     <row r="54" spans="4:13">
@@ -4411,21 +4284,21 @@
         <v>51</v>
       </c>
       <c r="E54" s="35" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="F54" s="34"/>
       <c r="H54" s="34">
         <v>51</v>
       </c>
       <c r="I54" s="35" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="J54" s="34"/>
       <c r="L54" s="34">
         <v>51</v>
       </c>
       <c r="M54" s="35" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="55" spans="4:13">
@@ -4433,14 +4306,14 @@
         <v>52</v>
       </c>
       <c r="E55" s="35" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="F55" s="34"/>
       <c r="L55" s="34">
         <v>52</v>
       </c>
       <c r="M55" s="35" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
     </row>
     <row r="56" spans="4:13">
@@ -4448,14 +4321,14 @@
         <v>53</v>
       </c>
       <c r="E56" s="35" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="F56" s="34"/>
       <c r="L56" s="34">
         <v>53</v>
       </c>
       <c r="M56" s="35" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
     </row>
     <row r="57" spans="4:13">
@@ -4463,14 +4336,14 @@
         <v>54</v>
       </c>
       <c r="E57" s="35" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="F57" s="34"/>
       <c r="L57" s="34">
         <v>54</v>
       </c>
       <c r="M57" s="35" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
     </row>
     <row r="58" spans="4:13">
@@ -4478,14 +4351,14 @@
         <v>55</v>
       </c>
       <c r="E58" s="35" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="F58" s="34"/>
       <c r="L58" s="34">
         <v>55</v>
       </c>
       <c r="M58" s="35" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
     </row>
     <row r="59" spans="4:13">
@@ -4493,14 +4366,14 @@
         <v>56</v>
       </c>
       <c r="E59" s="35" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="F59" s="34"/>
       <c r="L59" s="34">
         <v>56</v>
       </c>
       <c r="M59" s="35" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
     </row>
     <row r="60" spans="4:13">
@@ -4508,14 +4381,14 @@
         <v>57</v>
       </c>
       <c r="E60" s="35" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="F60" s="34"/>
       <c r="L60" s="34">
         <v>57</v>
       </c>
       <c r="M60" s="35" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
     </row>
     <row r="61" spans="4:13">
@@ -4523,14 +4396,14 @@
         <v>58</v>
       </c>
       <c r="E61" s="35" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="F61" s="34"/>
       <c r="L61" s="34">
         <v>58</v>
       </c>
       <c r="M61" s="35" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
     </row>
     <row r="62" spans="4:13">
@@ -4538,14 +4411,14 @@
         <v>59</v>
       </c>
       <c r="E62" s="35" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="F62" s="34"/>
       <c r="L62" s="34">
         <v>59</v>
       </c>
       <c r="M62" s="35" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
     </row>
     <row r="63" spans="4:13">
@@ -4553,14 +4426,14 @@
         <v>60</v>
       </c>
       <c r="E63" s="35" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="F63" s="34"/>
       <c r="L63" s="34">
         <v>60</v>
       </c>
       <c r="M63" s="35" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
     </row>
     <row r="64" spans="4:13">
@@ -4568,14 +4441,14 @@
         <v>61</v>
       </c>
       <c r="E64" s="35" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="F64" s="34"/>
       <c r="L64" s="34">
         <v>61</v>
       </c>
       <c r="M64" s="35" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
     </row>
     <row r="65" spans="4:13">
@@ -4583,14 +4456,14 @@
         <v>62</v>
       </c>
       <c r="E65" s="35" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="F65" s="34"/>
       <c r="L65" s="34">
         <v>62</v>
       </c>
       <c r="M65" s="35" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
     </row>
     <row r="66" spans="4:13">
@@ -4598,14 +4471,14 @@
         <v>63</v>
       </c>
       <c r="E66" s="35" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
       <c r="F66" s="34"/>
       <c r="L66" s="34">
         <v>63</v>
       </c>
       <c r="M66" s="35" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
     </row>
     <row r="67" spans="4:13">
@@ -4613,14 +4486,14 @@
         <v>64</v>
       </c>
       <c r="E67" s="35" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="F67" s="34"/>
       <c r="L67" s="34">
         <v>64</v>
       </c>
       <c r="M67" s="35" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
     </row>
     <row r="68" spans="4:13">
@@ -4628,14 +4501,14 @@
         <v>65</v>
       </c>
       <c r="E68" s="35" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="F68" s="34"/>
       <c r="L68" s="34">
         <v>65</v>
       </c>
       <c r="M68" s="35" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
     </row>
     <row r="69" spans="4:13">
@@ -4643,14 +4516,14 @@
         <v>66</v>
       </c>
       <c r="E69" s="35" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="F69" s="34"/>
       <c r="L69" s="34">
         <v>66</v>
       </c>
       <c r="M69" s="35" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
     </row>
     <row r="70" spans="4:13">
@@ -4658,14 +4531,14 @@
         <v>67</v>
       </c>
       <c r="E70" s="35" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="F70" s="34"/>
       <c r="L70" s="34">
         <v>67</v>
       </c>
       <c r="M70" s="35" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
     </row>
     <row r="71" spans="4:13">
@@ -4673,14 +4546,14 @@
         <v>68</v>
       </c>
       <c r="E71" s="35" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="F71" s="34"/>
       <c r="L71" s="34">
         <v>68</v>
       </c>
       <c r="M71" s="35" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
     </row>
     <row r="72" spans="4:13">
@@ -4688,14 +4561,14 @@
         <v>69</v>
       </c>
       <c r="E72" s="35" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="F72" s="34"/>
       <c r="L72" s="34">
         <v>69</v>
       </c>
       <c r="M72" s="35" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
     </row>
     <row r="73" spans="4:13">
@@ -4703,14 +4576,14 @@
         <v>70</v>
       </c>
       <c r="E73" s="35" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
       <c r="F73" s="34"/>
       <c r="L73" s="34">
         <v>70</v>
       </c>
       <c r="M73" s="35" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
     </row>
     <row r="74" spans="4:13">
@@ -4718,14 +4591,14 @@
         <v>71</v>
       </c>
       <c r="E74" s="35" t="s">
-        <v>347</v>
+        <v>336</v>
       </c>
       <c r="F74" s="34"/>
       <c r="L74" s="34">
         <v>71</v>
       </c>
       <c r="M74" s="35" t="s">
-        <v>348</v>
+        <v>337</v>
       </c>
     </row>
     <row r="75" spans="4:13">
@@ -4733,14 +4606,14 @@
         <v>72</v>
       </c>
       <c r="E75" s="35" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="F75" s="34"/>
       <c r="L75" s="34">
         <v>72</v>
       </c>
       <c r="M75" s="35" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
     </row>
     <row r="76" spans="4:13">
@@ -4748,14 +4621,14 @@
         <v>73</v>
       </c>
       <c r="E76" s="35" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F76" s="34"/>
       <c r="L76" s="34">
         <v>73</v>
       </c>
       <c r="M76" s="35" t="s">
-        <v>352</v>
+        <v>341</v>
       </c>
     </row>
     <row r="77" spans="4:13">
@@ -4763,14 +4636,14 @@
         <v>74</v>
       </c>
       <c r="E77" s="35" t="s">
-        <v>353</v>
+        <v>342</v>
       </c>
       <c r="F77" s="34"/>
       <c r="L77" s="34">
         <v>74</v>
       </c>
       <c r="M77" s="35" t="s">
-        <v>354</v>
+        <v>343</v>
       </c>
     </row>
     <row r="78" spans="4:13">
@@ -4778,14 +4651,14 @@
         <v>75</v>
       </c>
       <c r="E78" s="35" t="s">
-        <v>355</v>
+        <v>344</v>
       </c>
       <c r="F78" s="34"/>
       <c r="L78" s="34">
         <v>75</v>
       </c>
       <c r="M78" s="35" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
     </row>
     <row r="79" spans="4:13">
@@ -4793,7 +4666,7 @@
         <v>76</v>
       </c>
       <c r="E79" s="35" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="F79" s="34"/>
     </row>
@@ -4802,7 +4675,7 @@
         <v>77</v>
       </c>
       <c r="E80" s="35" t="s">
-        <v>358</v>
+        <v>347</v>
       </c>
       <c r="F80" s="34"/>
     </row>
@@ -4811,7 +4684,7 @@
         <v>78</v>
       </c>
       <c r="E81" s="35" t="s">
-        <v>359</v>
+        <v>348</v>
       </c>
       <c r="F81" s="34"/>
     </row>
@@ -4820,7 +4693,7 @@
         <v>79</v>
       </c>
       <c r="E82" s="35" t="s">
-        <v>360</v>
+        <v>349</v>
       </c>
       <c r="F82" s="34"/>
     </row>
@@ -4829,7 +4702,7 @@
         <v>80</v>
       </c>
       <c r="E83" s="35" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F83" s="34"/>
     </row>
@@ -4838,7 +4711,7 @@
         <v>81</v>
       </c>
       <c r="E84" s="35" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="F84" s="34"/>
     </row>
@@ -4847,7 +4720,7 @@
         <v>82</v>
       </c>
       <c r="E85" s="35" t="s">
-        <v>363</v>
+        <v>352</v>
       </c>
       <c r="F85" s="34"/>
     </row>
@@ -4856,7 +4729,7 @@
         <v>83</v>
       </c>
       <c r="E86" s="35" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="F86" s="34"/>
     </row>
@@ -4865,7 +4738,7 @@
         <v>84</v>
       </c>
       <c r="E87" s="35" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="F87" s="34"/>
     </row>
@@ -4874,7 +4747,7 @@
         <v>85</v>
       </c>
       <c r="E88" s="35" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="F88" s="34"/>
     </row>
@@ -4883,7 +4756,7 @@
         <v>86</v>
       </c>
       <c r="E89" s="35" t="s">
-        <v>367</v>
+        <v>356</v>
       </c>
       <c r="F89" s="34"/>
     </row>
@@ -4892,7 +4765,7 @@
         <v>87</v>
       </c>
       <c r="E90" s="35" t="s">
-        <v>368</v>
+        <v>357</v>
       </c>
       <c r="F90" s="34"/>
     </row>
@@ -4901,7 +4774,7 @@
         <v>88</v>
       </c>
       <c r="E91" s="35" t="s">
-        <v>369</v>
+        <v>358</v>
       </c>
       <c r="F91" s="34"/>
     </row>
@@ -4910,7 +4783,7 @@
         <v>89</v>
       </c>
       <c r="E92" s="35" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="F92" s="34"/>
     </row>
@@ -4919,7 +4792,7 @@
         <v>90</v>
       </c>
       <c r="E93" s="35" t="s">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="F93" s="34"/>
     </row>
@@ -4928,7 +4801,7 @@
         <v>91</v>
       </c>
       <c r="E94" s="35" t="s">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="F94" s="34"/>
     </row>
@@ -4937,7 +4810,7 @@
         <v>92</v>
       </c>
       <c r="E95" s="35" t="s">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="F95" s="34"/>
     </row>
@@ -4946,7 +4819,7 @@
         <v>93</v>
       </c>
       <c r="E96" s="35" t="s">
-        <v>373</v>
+        <v>362</v>
       </c>
       <c r="F96" s="34"/>
     </row>
@@ -4955,7 +4828,7 @@
         <v>94</v>
       </c>
       <c r="E97" s="35" t="s">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="F97" s="34"/>
     </row>
@@ -4964,7 +4837,7 @@
         <v>95</v>
       </c>
       <c r="E98" s="35" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="F98" s="34"/>
     </row>
@@ -4973,7 +4846,7 @@
         <v>96</v>
       </c>
       <c r="E99" s="35" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
       <c r="F99" s="34"/>
     </row>
@@ -4982,7 +4855,7 @@
         <v>97</v>
       </c>
       <c r="E100" s="35" t="s">
-        <v>377</v>
+        <v>366</v>
       </c>
       <c r="F100" s="34"/>
     </row>
@@ -4991,7 +4864,7 @@
         <v>98</v>
       </c>
       <c r="E101" s="35" t="s">
-        <v>378</v>
+        <v>367</v>
       </c>
       <c r="F101" s="34"/>
     </row>
@@ -5000,7 +4873,7 @@
         <v>99</v>
       </c>
       <c r="E102" s="35" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
       <c r="F102" s="34"/>
     </row>
@@ -5009,7 +4882,7 @@
         <v>100</v>
       </c>
       <c r="E103" s="35" t="s">
-        <v>380</v>
+        <v>369</v>
       </c>
       <c r="F103" s="34"/>
     </row>
@@ -5018,7 +4891,7 @@
         <v>101</v>
       </c>
       <c r="E104" s="35" t="s">
-        <v>381</v>
+        <v>370</v>
       </c>
       <c r="F104" s="34"/>
     </row>
@@ -5027,7 +4900,7 @@
         <v>102</v>
       </c>
       <c r="E105" s="35" t="s">
-        <v>382</v>
+        <v>371</v>
       </c>
       <c r="F105" s="34"/>
     </row>
@@ -5036,7 +4909,7 @@
         <v>103</v>
       </c>
       <c r="E106" s="35" t="s">
-        <v>383</v>
+        <v>372</v>
       </c>
       <c r="F106" s="34"/>
     </row>
@@ -5045,7 +4918,7 @@
         <v>104</v>
       </c>
       <c r="E107" s="35" t="s">
-        <v>384</v>
+        <v>373</v>
       </c>
       <c r="F107" s="34"/>
     </row>
@@ -5054,7 +4927,7 @@
         <v>105</v>
       </c>
       <c r="E108" s="35" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="F108" s="34"/>
     </row>
@@ -5063,7 +4936,7 @@
         <v>106</v>
       </c>
       <c r="E109" s="35" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="F109" s="34"/>
     </row>
@@ -5072,7 +4945,7 @@
         <v>107</v>
       </c>
       <c r="E110" s="35" t="s">
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="F110" s="34"/>
     </row>
@@ -5081,7 +4954,7 @@
         <v>108</v>
       </c>
       <c r="E111" s="35" t="s">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="F111" s="34"/>
     </row>
@@ -5090,7 +4963,7 @@
         <v>109</v>
       </c>
       <c r="E112" s="35" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="F112" s="34"/>
     </row>
@@ -5099,7 +4972,7 @@
         <v>110</v>
       </c>
       <c r="E113" s="35" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="F113" s="34"/>
     </row>
@@ -5108,7 +4981,7 @@
         <v>111</v>
       </c>
       <c r="E114" s="35" t="s">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="F114" s="34"/>
     </row>
@@ -5117,7 +4990,7 @@
         <v>112</v>
       </c>
       <c r="E115" s="35" t="s">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="F115" s="34"/>
     </row>
@@ -5126,7 +4999,7 @@
         <v>113</v>
       </c>
       <c r="E116" s="35" t="s">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="F116" s="34"/>
     </row>
@@ -5135,7 +5008,7 @@
         <v>114</v>
       </c>
       <c r="E117" s="35" t="s">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="F117" s="34"/>
     </row>
@@ -5144,7 +5017,7 @@
         <v>115</v>
       </c>
       <c r="E118" s="35" t="s">
-        <v>395</v>
+        <v>384</v>
       </c>
       <c r="F118" s="34"/>
     </row>
@@ -5153,7 +5026,7 @@
         <v>116</v>
       </c>
       <c r="E119" s="35" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="F119" s="34"/>
     </row>
@@ -5162,7 +5035,7 @@
         <v>117</v>
       </c>
       <c r="E120" s="35" t="s">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="F120" s="34"/>
     </row>
@@ -5171,7 +5044,7 @@
         <v>118</v>
       </c>
       <c r="E121" s="35" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="F121" s="34"/>
     </row>
@@ -5180,7 +5053,7 @@
         <v>119</v>
       </c>
       <c r="E122" s="35" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
       <c r="F122" s="34"/>
     </row>
@@ -5189,7 +5062,7 @@
         <v>120</v>
       </c>
       <c r="E123" s="35" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="F123" s="34"/>
     </row>
@@ -5198,7 +5071,7 @@
         <v>121</v>
       </c>
       <c r="E124" s="35" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="F124" s="34"/>
     </row>
@@ -5207,7 +5080,7 @@
         <v>122</v>
       </c>
       <c r="E125" s="35" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="F125" s="34"/>
     </row>
@@ -5216,7 +5089,7 @@
         <v>123</v>
       </c>
       <c r="E126" s="35" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="F126" s="34"/>
     </row>
@@ -5225,7 +5098,7 @@
         <v>124</v>
       </c>
       <c r="E127" s="35" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="F127" s="34"/>
     </row>
@@ -5234,7 +5107,7 @@
         <v>125</v>
       </c>
       <c r="E128" s="35" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="F128" s="34"/>
     </row>
@@ -5243,7 +5116,7 @@
         <v>126</v>
       </c>
       <c r="E129" s="35" t="s">
-        <v>406</v>
+        <v>395</v>
       </c>
       <c r="F129" s="34"/>
     </row>
@@ -5252,7 +5125,7 @@
         <v>127</v>
       </c>
       <c r="E130" s="35" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="F130" s="34"/>
     </row>
@@ -5261,7 +5134,7 @@
         <v>128</v>
       </c>
       <c r="E131" s="35" t="s">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="F131" s="34"/>
     </row>
@@ -5270,7 +5143,7 @@
         <v>129</v>
       </c>
       <c r="E132" s="35" t="s">
-        <v>409</v>
+        <v>398</v>
       </c>
       <c r="F132" s="34"/>
     </row>
@@ -5279,7 +5152,7 @@
         <v>130</v>
       </c>
       <c r="E133" s="35" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="F133" s="34"/>
     </row>
@@ -5288,7 +5161,7 @@
         <v>131</v>
       </c>
       <c r="E134" s="35" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="F134" s="34"/>
     </row>
@@ -5297,7 +5170,7 @@
         <v>132</v>
       </c>
       <c r="E135" s="35" t="s">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="F135" s="34"/>
     </row>
@@ -5306,7 +5179,7 @@
         <v>133</v>
       </c>
       <c r="E136" s="35" t="s">
-        <v>413</v>
+        <v>402</v>
       </c>
       <c r="F136" s="34"/>
     </row>
@@ -5315,7 +5188,7 @@
         <v>134</v>
       </c>
       <c r="E137" s="35" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="F137" s="34"/>
     </row>
@@ -5324,7 +5197,7 @@
         <v>135</v>
       </c>
       <c r="E138" s="35" t="s">
-        <v>415</v>
+        <v>404</v>
       </c>
       <c r="F138" s="34"/>
     </row>
@@ -5333,7 +5206,7 @@
         <v>136</v>
       </c>
       <c r="E139" s="35" t="s">
-        <v>416</v>
+        <v>405</v>
       </c>
       <c r="F139" s="34"/>
     </row>
@@ -5342,7 +5215,7 @@
         <v>137</v>
       </c>
       <c r="E140" s="35" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="F140" s="34"/>
     </row>
@@ -5351,7 +5224,7 @@
         <v>138</v>
       </c>
       <c r="E141" s="35" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="F141" s="34"/>
     </row>
@@ -5360,7 +5233,7 @@
         <v>139</v>
       </c>
       <c r="E142" s="35" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="F142" s="34"/>
     </row>
@@ -5369,7 +5242,7 @@
         <v>140</v>
       </c>
       <c r="E143" s="35" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
       <c r="F143" s="34"/>
     </row>
@@ -5378,7 +5251,7 @@
         <v>141</v>
       </c>
       <c r="E144" s="35" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="F144" s="34"/>
     </row>
@@ -5387,7 +5260,7 @@
         <v>142</v>
       </c>
       <c r="E145" s="35" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="F145" s="34"/>
     </row>
@@ -5396,7 +5269,7 @@
         <v>143</v>
       </c>
       <c r="E146" s="35" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="F146" s="34"/>
     </row>
@@ -5405,7 +5278,7 @@
         <v>144</v>
       </c>
       <c r="E147" s="35" t="s">
-        <v>424</v>
+        <v>413</v>
       </c>
       <c r="F147" s="34"/>
     </row>
@@ -5414,7 +5287,7 @@
         <v>145</v>
       </c>
       <c r="E148" s="35" t="s">
-        <v>425</v>
+        <v>414</v>
       </c>
       <c r="F148" s="34"/>
     </row>
@@ -5423,7 +5296,7 @@
         <v>146</v>
       </c>
       <c r="E149" s="35" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
       <c r="F149" s="34"/>
     </row>
@@ -5432,7 +5305,7 @@
         <v>147</v>
       </c>
       <c r="E150" s="35" t="s">
-        <v>427</v>
+        <v>416</v>
       </c>
       <c r="F150" s="34"/>
     </row>
@@ -5441,7 +5314,7 @@
         <v>148</v>
       </c>
       <c r="E151" s="35" t="s">
-        <v>428</v>
+        <v>417</v>
       </c>
       <c r="F151" s="34"/>
     </row>
@@ -5450,7 +5323,7 @@
         <v>149</v>
       </c>
       <c r="E152" s="35" t="s">
-        <v>429</v>
+        <v>418</v>
       </c>
       <c r="F152" s="34"/>
     </row>
@@ -5459,7 +5332,7 @@
         <v>150</v>
       </c>
       <c r="E153" s="35" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
       <c r="F153" s="34"/>
     </row>
@@ -5468,7 +5341,7 @@
         <v>151</v>
       </c>
       <c r="E154" s="35" t="s">
-        <v>431</v>
+        <v>420</v>
       </c>
       <c r="F154" s="34"/>
     </row>
@@ -5477,7 +5350,7 @@
         <v>152</v>
       </c>
       <c r="E155" s="35" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
       <c r="F155" s="34"/>
     </row>
@@ -5486,7 +5359,7 @@
         <v>153</v>
       </c>
       <c r="E156" s="35" t="s">
-        <v>433</v>
+        <v>422</v>
       </c>
       <c r="F156" s="34"/>
     </row>
@@ -5495,7 +5368,7 @@
         <v>154</v>
       </c>
       <c r="E157" s="35" t="s">
-        <v>434</v>
+        <v>423</v>
       </c>
       <c r="F157" s="34"/>
     </row>
@@ -5504,7 +5377,7 @@
         <v>155</v>
       </c>
       <c r="E158" s="35" t="s">
-        <v>435</v>
+        <v>424</v>
       </c>
       <c r="F158" s="34"/>
     </row>
@@ -5513,7 +5386,7 @@
         <v>156</v>
       </c>
       <c r="E159" s="35" t="s">
-        <v>436</v>
+        <v>425</v>
       </c>
       <c r="F159" s="34"/>
     </row>
@@ -5522,7 +5395,7 @@
         <v>157</v>
       </c>
       <c r="E160" s="35" t="s">
-        <v>437</v>
+        <v>426</v>
       </c>
       <c r="F160" s="34"/>
     </row>
@@ -5531,7 +5404,7 @@
         <v>158</v>
       </c>
       <c r="E161" s="35" t="s">
-        <v>438</v>
+        <v>427</v>
       </c>
       <c r="F161" s="34"/>
     </row>
@@ -5540,7 +5413,7 @@
         <v>159</v>
       </c>
       <c r="E162" s="35" t="s">
-        <v>439</v>
+        <v>428</v>
       </c>
       <c r="F162" s="34"/>
     </row>

</xml_diff>